<commit_message>
Expand sample documents with richer content for better RAG retrieval
</commit_message>
<xml_diff>
--- a/data/sample_docs/training_records.xlsx
+++ b/data/sample_docs/training_records.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="TrainingRecords" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CourseCatalog" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,31 +426,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>employee_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>department</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>course_name</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>completion_status</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>score</t>
         </is>
@@ -468,11 +481,11 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -486,16 +499,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>88</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1003</v>
+        <v>1001</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -509,44 +522,44 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1004</v>
+        <v>1002</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Customer Communication</t>
+          <t>Data Privacy</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1005</v>
+        <v>1002</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Safety Compliance</t>
+          <t>Security Awareness</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -556,6 +569,697 @@
       </c>
       <c r="E6" t="n">
         <v>90</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1002</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Insider Threat Prevention</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1003</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Security Awareness</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1003</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1003</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Secure Coding Practices</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1004</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Customer Communication</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1004</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Workplace Ethics</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>1004</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Security Awareness</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1005</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Safety Compliance</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>1005</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Security Awareness</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>1005</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Workplace Ethics</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>1006</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Secure Coding Practices</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>1006</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Security Awareness</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>1006</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>1007</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Secure Coding Practices</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>1007</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Security Awareness</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>1008</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Workplace Ethics</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>1008</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>1008</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Security Awareness</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>1009</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Customer Communication</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>1009</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Security Awareness</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>1009</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>1010</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Safety Compliance</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>1010</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Security Awareness</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>course_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>duration_hours</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>frequency</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>passing_score</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Security Awareness</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Workplace Ethics</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Biennial</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Safety Compliance</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Customer Communication</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>One-time</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Secure Coding Practices</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Insider Threat Prevention</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>